<commit_message>
All Modules tested with 0 failures
</commit_message>
<xml_diff>
--- a/src/test/resources/Checkout_YourInfo_TestData.xlsx
+++ b/src/test/resources/Checkout_YourInfo_TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{ECE258BC-C1E0-404C-80E5-0224AE17E318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{27D562C5-4BFB-4AC2-BA5A-E2996E45A77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Positive Test Cases" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="13">
   <si>
     <t>FirstName</t>
   </si>
@@ -38,36 +38,12 @@
     <t>560001</t>
   </si>
   <si>
-    <t>Donald</t>
-  </si>
-  <si>
     <t>Duck</t>
   </si>
   <si>
     <t>Tom</t>
   </si>
   <si>
-    <t>Cat</t>
-  </si>
-  <si>
-    <t>560002</t>
-  </si>
-  <si>
-    <t>Jerry</t>
-  </si>
-  <si>
-    <t>560003</t>
-  </si>
-  <si>
-    <t>Scooby</t>
-  </si>
-  <si>
-    <t>Doo</t>
-  </si>
-  <si>
-    <t>560004</t>
-  </si>
-  <si>
     <t>Bugs</t>
   </si>
   <si>
@@ -77,55 +53,10 @@
     <t>560005</t>
   </si>
   <si>
-    <t>Dora</t>
-  </si>
-  <si>
-    <t>Explorer</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Popeye</t>
-  </si>
-  <si>
-    <t>Sailor</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>ABCDE</t>
-  </si>
-  <si>
-    <t>12AB</t>
-  </si>
-  <si>
-    <t>Tom123</t>
-  </si>
-  <si>
-    <t>Jerry456</t>
-  </si>
-  <si>
-    <t>12345678901234567890</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
     <t>Mickeyyyyyyyyyyyyyyyyyyyyy</t>
   </si>
   <si>
-    <t>C</t>
-  </si>
-  <si>
     <t>Mouseeeeeeeeeeeeeeeeeeeee</t>
-  </si>
-  <si>
-    <t>999999</t>
-  </si>
-  <si>
-    <t>1000000</t>
   </si>
 </sst>
 </file>
@@ -476,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -505,83 +436,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
+    <row r="4" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -610,7 +482,7 @@
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>5</v>
@@ -618,104 +490,30 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="2"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
+        <v>9</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -741,105 +539,35 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
+    <row r="4" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
All bugs fixed and maintained clean code
</commit_message>
<xml_diff>
--- a/src/test/resources/Checkout_YourInfo_TestData.xlsx
+++ b/src/test/resources/Checkout_YourInfo_TestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{27D562C5-4BFB-4AC2-BA5A-E2996E45A77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{4FA4448E-20A8-421B-8320-8E6A8F85A380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Positive Test Cases" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Boundary Test Cases" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:P8"/>
+  <oleSize ref="A1:Q10"/>
 </workbook>
 </file>
 
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -436,7 +436,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -447,13 +447,6 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -461,7 +454,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -497,7 +490,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -506,14 +499,6 @@
       </c>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -521,7 +506,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -539,7 +524,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -550,7 +535,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -561,13 +546,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:3" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>